<commit_message>
Added WIP SRNTGT006 Updated Target folder list with existing folders
</commit_message>
<xml_diff>
--- a/INTEL/OPAC_JOINT_TARGET_LIST_v 0.2.xlsx
+++ b/INTEL/OPAC_JOINT_TARGET_LIST_v 0.2.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\GitHub\OPAT-background\INTEL\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olahe\Git-projects\OPAT-background\INTEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34A24BEC-A863-468C-AF7E-531A973418B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AABCA29-E4A3-42F3-8DC1-EC117C32AD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="840" yWindow="-120" windowWidth="37680" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="OPAC Joint Target List" sheetId="1" r:id="rId1"/>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1405" uniqueCount="911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="911">
   <si>
     <t>OPERATION ARCTIC CITADEL JOINT TARGET LIST</t>
   </si>
@@ -3894,25 +3894,20 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3926,17 +3921,22 @@
     <xf numFmtId="0" fontId="17" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -3945,18 +3945,18 @@
     <xf numFmtId="0" fontId="23" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="24" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normál" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -5410,7 +5410,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="11.625" customWidth="1"/>
     <col min="2" max="2" width="34.375" customWidth="1"/>
@@ -5446,7 +5446,7 @@
       </c>
       <c r="K1" s="3"/>
     </row>
-    <row r="2" spans="1:11" ht="45.75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" ht="34.5" x14ac:dyDescent="0.25">
       <c r="A2" s="142" t="s">
         <v>4</v>
       </c>
@@ -5910,7 +5910,9 @@
       <c r="I16" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J16" s="9"/>
+      <c r="J16" s="24" t="s">
+        <v>22</v>
+      </c>
       <c r="K16" s="3" t="s">
         <v>29</v>
       </c>
@@ -5941,7 +5943,9 @@
       <c r="I17" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J17" s="9"/>
+      <c r="J17" s="24" t="s">
+        <v>22</v>
+      </c>
       <c r="K17" s="3" t="s">
         <v>29</v>
       </c>
@@ -8595,7 +8599,9 @@
       <c r="I97" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J97" s="9"/>
+      <c r="J97" s="24" t="s">
+        <v>22</v>
+      </c>
       <c r="K97" s="3" t="s">
         <v>29</v>
       </c>
@@ -16280,7 +16286,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:Q1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="6.75" customWidth="1"/>
     <col min="2" max="2" width="11.5" customWidth="1"/>
@@ -16295,50 +16301,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="144" t="s">
+      <c r="A1" s="159" t="s">
         <v>759</v>
       </c>
-      <c r="B1" s="145"/>
-      <c r="C1" s="145"/>
-      <c r="D1" s="145"/>
-      <c r="E1" s="145"/>
-      <c r="F1" s="145"/>
-      <c r="G1" s="145"/>
-      <c r="H1" s="145"/>
-      <c r="I1" s="146"/>
+      <c r="B1" s="160"/>
+      <c r="C1" s="160"/>
+      <c r="D1" s="160"/>
+      <c r="E1" s="160"/>
+      <c r="F1" s="160"/>
+      <c r="G1" s="160"/>
+      <c r="H1" s="160"/>
+      <c r="I1" s="161"/>
     </row>
     <row r="2" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="147" t="s">
+      <c r="A2" s="162" t="s">
         <v>760</v>
       </c>
-      <c r="B2" s="148"/>
+      <c r="B2" s="147"/>
       <c r="C2" s="86" t="s">
         <v>761</v>
       </c>
-      <c r="D2" s="149" t="s">
+      <c r="D2" s="163" t="s">
         <v>762</v>
       </c>
       <c r="E2" s="150"/>
       <c r="F2" s="150"/>
-      <c r="G2" s="148"/>
-      <c r="H2" s="151" t="s">
+      <c r="G2" s="147"/>
+      <c r="H2" s="164" t="s">
         <v>763</v>
       </c>
-      <c r="I2" s="152"/>
+      <c r="I2" s="151"/>
     </row>
     <row r="3" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="153" t="s">
+      <c r="A4" s="165" t="s">
         <v>764</v>
       </c>
-      <c r="B4" s="145"/>
-      <c r="C4" s="145"/>
-      <c r="D4" s="145"/>
-      <c r="E4" s="145"/>
-      <c r="F4" s="145"/>
-      <c r="G4" s="145"/>
-      <c r="H4" s="145"/>
-      <c r="I4" s="146"/>
+      <c r="B4" s="160"/>
+      <c r="C4" s="160"/>
+      <c r="D4" s="160"/>
+      <c r="E4" s="160"/>
+      <c r="F4" s="160"/>
+      <c r="G4" s="160"/>
+      <c r="H4" s="160"/>
+      <c r="I4" s="161"/>
     </row>
     <row r="5" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="87" t="s">
@@ -16400,15 +16406,15 @@
       <c r="I6" s="92" t="s">
         <v>781</v>
       </c>
-      <c r="K6" s="154" t="s">
+      <c r="K6" s="153" t="s">
         <v>782</v>
       </c>
-      <c r="L6" s="155"/>
-      <c r="M6" s="155"/>
-      <c r="N6" s="155"/>
-      <c r="O6" s="155"/>
-      <c r="P6" s="155"/>
-      <c r="Q6" s="155"/>
+      <c r="L6" s="154"/>
+      <c r="M6" s="154"/>
+      <c r="N6" s="154"/>
+      <c r="O6" s="154"/>
+      <c r="P6" s="154"/>
+      <c r="Q6" s="154"/>
     </row>
     <row r="7" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="90">
@@ -16438,15 +16444,15 @@
       <c r="I7" s="92" t="s">
         <v>790</v>
       </c>
-      <c r="K7" s="154" t="s">
+      <c r="K7" s="153" t="s">
         <v>791</v>
       </c>
-      <c r="L7" s="155"/>
-      <c r="M7" s="155"/>
-      <c r="N7" s="155"/>
-      <c r="O7" s="155"/>
-      <c r="P7" s="155"/>
-      <c r="Q7" s="155"/>
+      <c r="L7" s="154"/>
+      <c r="M7" s="154"/>
+      <c r="N7" s="154"/>
+      <c r="O7" s="154"/>
+      <c r="P7" s="154"/>
+      <c r="Q7" s="154"/>
     </row>
     <row r="8" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="90">
@@ -16554,17 +16560,17 @@
       <c r="I14" s="81"/>
     </row>
     <row r="15" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="156" t="s">
+      <c r="A15" s="155" t="s">
         <v>800</v>
       </c>
-      <c r="B15" s="157"/>
-      <c r="C15" s="157"/>
-      <c r="D15" s="157"/>
-      <c r="E15" s="157"/>
-      <c r="F15" s="157"/>
-      <c r="G15" s="157"/>
-      <c r="H15" s="157"/>
-      <c r="I15" s="158"/>
+      <c r="B15" s="156"/>
+      <c r="C15" s="156"/>
+      <c r="D15" s="156"/>
+      <c r="E15" s="156"/>
+      <c r="F15" s="156"/>
+      <c r="G15" s="156"/>
+      <c r="H15" s="156"/>
+      <c r="I15" s="157"/>
     </row>
     <row r="16" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="87" t="s">
@@ -16579,15 +16585,15 @@
       <c r="D16" s="88" t="s">
         <v>772</v>
       </c>
-      <c r="E16" s="159" t="s">
+      <c r="E16" s="158" t="s">
         <v>801</v>
       </c>
-      <c r="F16" s="160"/>
-      <c r="G16" s="159" t="s">
+      <c r="F16" s="145"/>
+      <c r="G16" s="158" t="s">
         <v>802</v>
       </c>
-      <c r="H16" s="161"/>
-      <c r="I16" s="162"/>
+      <c r="H16" s="148"/>
+      <c r="I16" s="149"/>
     </row>
     <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="96">
@@ -16602,15 +16608,15 @@
       <c r="D17" s="91" t="s">
         <v>799</v>
       </c>
-      <c r="E17" s="163" t="s">
+      <c r="E17" s="152" t="s">
         <v>804</v>
       </c>
-      <c r="F17" s="160"/>
-      <c r="G17" s="163" t="s">
+      <c r="F17" s="145"/>
+      <c r="G17" s="152" t="s">
         <v>805</v>
       </c>
-      <c r="H17" s="161"/>
-      <c r="I17" s="162"/>
+      <c r="H17" s="148"/>
+      <c r="I17" s="149"/>
     </row>
     <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="96">
@@ -16625,15 +16631,15 @@
       <c r="D18" s="91" t="s">
         <v>799</v>
       </c>
-      <c r="E18" s="163" t="s">
+      <c r="E18" s="152" t="s">
         <v>804</v>
       </c>
-      <c r="F18" s="160"/>
-      <c r="G18" s="163" t="s">
+      <c r="F18" s="145"/>
+      <c r="G18" s="152" t="s">
         <v>807</v>
       </c>
-      <c r="H18" s="161"/>
-      <c r="I18" s="162"/>
+      <c r="H18" s="148"/>
+      <c r="I18" s="149"/>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="96">
@@ -16648,15 +16654,15 @@
       <c r="D19" s="91" t="s">
         <v>809</v>
       </c>
-      <c r="E19" s="163" t="s">
+      <c r="E19" s="152" t="s">
         <v>810</v>
       </c>
-      <c r="F19" s="160"/>
-      <c r="G19" s="163" t="s">
+      <c r="F19" s="145"/>
+      <c r="G19" s="152" t="s">
         <v>811</v>
       </c>
-      <c r="H19" s="161"/>
-      <c r="I19" s="162"/>
+      <c r="H19" s="148"/>
+      <c r="I19" s="149"/>
       <c r="K19" s="81" t="s">
         <v>812</v>
       </c>
@@ -16668,11 +16674,11 @@
       <c r="B20" s="97"/>
       <c r="C20" s="97"/>
       <c r="D20" s="97"/>
-      <c r="E20" s="164"/>
-      <c r="F20" s="160"/>
-      <c r="G20" s="164"/>
-      <c r="H20" s="161"/>
-      <c r="I20" s="162"/>
+      <c r="E20" s="144"/>
+      <c r="F20" s="145"/>
+      <c r="G20" s="144"/>
+      <c r="H20" s="148"/>
+      <c r="I20" s="149"/>
     </row>
     <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="96">
@@ -16681,11 +16687,11 @@
       <c r="B21" s="97"/>
       <c r="C21" s="97"/>
       <c r="D21" s="97"/>
-      <c r="E21" s="164"/>
-      <c r="F21" s="160"/>
-      <c r="G21" s="164"/>
-      <c r="H21" s="161"/>
-      <c r="I21" s="162"/>
+      <c r="E21" s="144"/>
+      <c r="F21" s="145"/>
+      <c r="G21" s="144"/>
+      <c r="H21" s="148"/>
+      <c r="I21" s="149"/>
       <c r="K21" s="81" t="s">
         <v>813</v>
       </c>
@@ -16697,11 +16703,11 @@
       <c r="B22" s="97"/>
       <c r="C22" s="97"/>
       <c r="D22" s="97"/>
-      <c r="E22" s="164"/>
-      <c r="F22" s="160"/>
-      <c r="G22" s="164"/>
-      <c r="H22" s="161"/>
-      <c r="I22" s="162"/>
+      <c r="E22" s="144"/>
+      <c r="F22" s="145"/>
+      <c r="G22" s="144"/>
+      <c r="H22" s="148"/>
+      <c r="I22" s="149"/>
     </row>
     <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="96">
@@ -16710,11 +16716,11 @@
       <c r="B23" s="97"/>
       <c r="C23" s="97"/>
       <c r="D23" s="97"/>
-      <c r="E23" s="164"/>
-      <c r="F23" s="160"/>
-      <c r="G23" s="164"/>
-      <c r="H23" s="161"/>
-      <c r="I23" s="162"/>
+      <c r="E23" s="144"/>
+      <c r="F23" s="145"/>
+      <c r="G23" s="144"/>
+      <c r="H23" s="148"/>
+      <c r="I23" s="149"/>
     </row>
     <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="96">
@@ -16723,11 +16729,11 @@
       <c r="B24" s="97"/>
       <c r="C24" s="97"/>
       <c r="D24" s="97"/>
-      <c r="E24" s="164"/>
-      <c r="F24" s="160"/>
-      <c r="G24" s="164"/>
-      <c r="H24" s="161"/>
-      <c r="I24" s="162"/>
+      <c r="E24" s="144"/>
+      <c r="F24" s="145"/>
+      <c r="G24" s="144"/>
+      <c r="H24" s="148"/>
+      <c r="I24" s="149"/>
     </row>
     <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="96">
@@ -16736,11 +16742,11 @@
       <c r="B25" s="97"/>
       <c r="C25" s="97"/>
       <c r="D25" s="97"/>
-      <c r="E25" s="164"/>
-      <c r="F25" s="160"/>
-      <c r="G25" s="164"/>
-      <c r="H25" s="161"/>
-      <c r="I25" s="162"/>
+      <c r="E25" s="144"/>
+      <c r="F25" s="145"/>
+      <c r="G25" s="144"/>
+      <c r="H25" s="148"/>
+      <c r="I25" s="149"/>
     </row>
     <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="98">
@@ -16749,11 +16755,11 @@
       <c r="B26" s="94"/>
       <c r="C26" s="94"/>
       <c r="D26" s="94"/>
-      <c r="E26" s="165"/>
-      <c r="F26" s="148"/>
-      <c r="G26" s="165"/>
+      <c r="E26" s="146"/>
+      <c r="F26" s="147"/>
+      <c r="G26" s="146"/>
       <c r="H26" s="150"/>
-      <c r="I26" s="152"/>
+      <c r="I26" s="151"/>
     </row>
     <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -17731,14 +17737,16 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="K7:Q7"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:I16"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:I17"/>
     <mergeCell ref="E18:F18"/>
@@ -17751,16 +17759,14 @@
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="G21:I21"/>
     <mergeCell ref="G22:I22"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="K7:Q7"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:I16"/>
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="A4:I4"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -17771,7 +17777,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:U1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="27" customWidth="1"/>
     <col min="2" max="2" width="27.375" customWidth="1"/>
@@ -19327,7 +19333,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="B1:O1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="11.625" customWidth="1"/>
@@ -19341,7 +19347,7 @@
       <c r="B2" s="168" t="s">
         <v>824</v>
       </c>
-      <c r="C2" s="160"/>
+      <c r="C2" s="145"/>
       <c r="O2" s="81" t="s">
         <v>825</v>
       </c>
@@ -20537,7 +20543,7 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:J1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="30.5" customWidth="1"/>
@@ -20555,53 +20561,53 @@
       <c r="A3" s="168" t="s">
         <v>857</v>
       </c>
-      <c r="B3" s="161"/>
-      <c r="C3" s="160"/>
+      <c r="B3" s="148"/>
+      <c r="C3" s="145"/>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="120" t="s">
         <v>765</v>
       </c>
-      <c r="B4" s="169" t="s">
+      <c r="B4" s="170" t="s">
         <v>858</v>
       </c>
-      <c r="C4" s="160"/>
+      <c r="C4" s="145"/>
     </row>
     <row r="5" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="121" t="s">
         <v>859</v>
       </c>
-      <c r="B5" s="170" t="s">
+      <c r="B5" s="169" t="s">
         <v>860</v>
       </c>
-      <c r="C5" s="160"/>
+      <c r="C5" s="145"/>
     </row>
     <row r="6" spans="1:10" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="121" t="s">
         <v>861</v>
       </c>
-      <c r="B6" s="170" t="s">
+      <c r="B6" s="169" t="s">
         <v>862</v>
       </c>
-      <c r="C6" s="160"/>
+      <c r="C6" s="145"/>
     </row>
     <row r="7" spans="1:10" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="121" t="s">
         <v>863</v>
       </c>
-      <c r="B7" s="170" t="s">
+      <c r="B7" s="169" t="s">
         <v>864</v>
       </c>
-      <c r="C7" s="160"/>
+      <c r="C7" s="145"/>
     </row>
     <row r="8" spans="1:10" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="121" t="s">
         <v>865</v>
       </c>
-      <c r="B8" s="170" t="s">
+      <c r="B8" s="169" t="s">
         <v>866</v>
       </c>
-      <c r="C8" s="160"/>
+      <c r="C8" s="145"/>
     </row>
     <row r="9" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -21613,7 +21619,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="B1:J1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="15.625" customWidth="1"/>
@@ -21629,8 +21635,8 @@
       <c r="B2" s="171" t="s">
         <v>867</v>
       </c>
-      <c r="C2" s="145"/>
-      <c r="D2" s="146"/>
+      <c r="C2" s="160"/>
+      <c r="D2" s="161"/>
       <c r="J2" s="81" t="s">
         <v>825</v>
       </c>
@@ -23154,7 +23160,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="C1:D1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="59.75" customWidth="1"/>
@@ -24192,7 +24198,7 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:J1000"/>
-  <sheetFormatPr defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.625" defaultRowHeight="15" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="30.5" customWidth="1"/>
@@ -24211,11 +24217,11 @@
     <row r="3" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="5" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="169" t="s">
+      <c r="A5" s="170" t="s">
         <v>900</v>
       </c>
-      <c r="B5" s="161"/>
-      <c r="C5" s="160"/>
+      <c r="B5" s="148"/>
+      <c r="C5" s="145"/>
     </row>
     <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="120" t="s">

</xml_diff>

<commit_message>
ADDED SRNTGT061 UPDATED TARGET LIST XLSX
</commit_message>
<xml_diff>
--- a/INTEL/OPAC_JOINT_TARGET_LIST_v 0.2.xlsx
+++ b/INTEL/OPAC_JOINT_TARGET_LIST_v 0.2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\olahe\Git-projects\OPAT-background\INTEL\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8AABCA29-E4A3-42F3-8DC1-EC117C32AD06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AFB68468-CB56-4426-B10B-F7F499E6CCDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1408" uniqueCount="911">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1409" uniqueCount="911">
   <si>
     <t>OPERATION ARCTIC CITADEL JOINT TARGET LIST</t>
   </si>
@@ -3894,20 +3894,25 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="26" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -3921,22 +3926,17 @@
     <xf numFmtId="0" fontId="17" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="10" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="7" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="24" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="9" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -7600,9 +7600,11 @@
       <c r="I64" s="24" t="s">
         <v>23</v>
       </c>
-      <c r="J64" s="9"/>
+      <c r="J64" s="24" t="s">
+        <v>22</v>
+      </c>
       <c r="K64" s="3" t="s">
-        <v>241</v>
+        <v>29</v>
       </c>
     </row>
     <row r="65" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -16301,50 +16303,50 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:17" ht="49.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="159" t="s">
+      <c r="A1" s="144" t="s">
         <v>759</v>
       </c>
-      <c r="B1" s="160"/>
-      <c r="C1" s="160"/>
-      <c r="D1" s="160"/>
-      <c r="E1" s="160"/>
-      <c r="F1" s="160"/>
-      <c r="G1" s="160"/>
-      <c r="H1" s="160"/>
-      <c r="I1" s="161"/>
+      <c r="B1" s="145"/>
+      <c r="C1" s="145"/>
+      <c r="D1" s="145"/>
+      <c r="E1" s="145"/>
+      <c r="F1" s="145"/>
+      <c r="G1" s="145"/>
+      <c r="H1" s="145"/>
+      <c r="I1" s="146"/>
     </row>
     <row r="2" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="162" t="s">
+      <c r="A2" s="147" t="s">
         <v>760</v>
       </c>
-      <c r="B2" s="147"/>
+      <c r="B2" s="148"/>
       <c r="C2" s="86" t="s">
         <v>761</v>
       </c>
-      <c r="D2" s="163" t="s">
+      <c r="D2" s="149" t="s">
         <v>762</v>
       </c>
       <c r="E2" s="150"/>
       <c r="F2" s="150"/>
-      <c r="G2" s="147"/>
-      <c r="H2" s="164" t="s">
+      <c r="G2" s="148"/>
+      <c r="H2" s="151" t="s">
         <v>763</v>
       </c>
-      <c r="I2" s="151"/>
+      <c r="I2" s="152"/>
     </row>
     <row r="3" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="4" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="165" t="s">
+      <c r="A4" s="153" t="s">
         <v>764</v>
       </c>
-      <c r="B4" s="160"/>
-      <c r="C4" s="160"/>
-      <c r="D4" s="160"/>
-      <c r="E4" s="160"/>
-      <c r="F4" s="160"/>
-      <c r="G4" s="160"/>
-      <c r="H4" s="160"/>
-      <c r="I4" s="161"/>
+      <c r="B4" s="145"/>
+      <c r="C4" s="145"/>
+      <c r="D4" s="145"/>
+      <c r="E4" s="145"/>
+      <c r="F4" s="145"/>
+      <c r="G4" s="145"/>
+      <c r="H4" s="145"/>
+      <c r="I4" s="146"/>
     </row>
     <row r="5" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="87" t="s">
@@ -16406,15 +16408,15 @@
       <c r="I6" s="92" t="s">
         <v>781</v>
       </c>
-      <c r="K6" s="153" t="s">
+      <c r="K6" s="154" t="s">
         <v>782</v>
       </c>
-      <c r="L6" s="154"/>
-      <c r="M6" s="154"/>
-      <c r="N6" s="154"/>
-      <c r="O6" s="154"/>
-      <c r="P6" s="154"/>
-      <c r="Q6" s="154"/>
+      <c r="L6" s="155"/>
+      <c r="M6" s="155"/>
+      <c r="N6" s="155"/>
+      <c r="O6" s="155"/>
+      <c r="P6" s="155"/>
+      <c r="Q6" s="155"/>
     </row>
     <row r="7" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="90">
@@ -16444,15 +16446,15 @@
       <c r="I7" s="92" t="s">
         <v>790</v>
       </c>
-      <c r="K7" s="153" t="s">
+      <c r="K7" s="154" t="s">
         <v>791</v>
       </c>
-      <c r="L7" s="154"/>
-      <c r="M7" s="154"/>
-      <c r="N7" s="154"/>
-      <c r="O7" s="154"/>
-      <c r="P7" s="154"/>
-      <c r="Q7" s="154"/>
+      <c r="L7" s="155"/>
+      <c r="M7" s="155"/>
+      <c r="N7" s="155"/>
+      <c r="O7" s="155"/>
+      <c r="P7" s="155"/>
+      <c r="Q7" s="155"/>
     </row>
     <row r="8" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="90">
@@ -16560,17 +16562,17 @@
       <c r="I14" s="81"/>
     </row>
     <row r="15" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="155" t="s">
+      <c r="A15" s="156" t="s">
         <v>800</v>
       </c>
-      <c r="B15" s="156"/>
-      <c r="C15" s="156"/>
-      <c r="D15" s="156"/>
-      <c r="E15" s="156"/>
-      <c r="F15" s="156"/>
-      <c r="G15" s="156"/>
-      <c r="H15" s="156"/>
-      <c r="I15" s="157"/>
+      <c r="B15" s="157"/>
+      <c r="C15" s="157"/>
+      <c r="D15" s="157"/>
+      <c r="E15" s="157"/>
+      <c r="F15" s="157"/>
+      <c r="G15" s="157"/>
+      <c r="H15" s="157"/>
+      <c r="I15" s="158"/>
     </row>
     <row r="16" spans="1:17" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A16" s="87" t="s">
@@ -16585,15 +16587,15 @@
       <c r="D16" s="88" t="s">
         <v>772</v>
       </c>
-      <c r="E16" s="158" t="s">
+      <c r="E16" s="159" t="s">
         <v>801</v>
       </c>
-      <c r="F16" s="145"/>
-      <c r="G16" s="158" t="s">
+      <c r="F16" s="160"/>
+      <c r="G16" s="159" t="s">
         <v>802</v>
       </c>
-      <c r="H16" s="148"/>
-      <c r="I16" s="149"/>
+      <c r="H16" s="161"/>
+      <c r="I16" s="162"/>
     </row>
     <row r="17" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A17" s="96">
@@ -16608,15 +16610,15 @@
       <c r="D17" s="91" t="s">
         <v>799</v>
       </c>
-      <c r="E17" s="152" t="s">
+      <c r="E17" s="163" t="s">
         <v>804</v>
       </c>
-      <c r="F17" s="145"/>
-      <c r="G17" s="152" t="s">
+      <c r="F17" s="160"/>
+      <c r="G17" s="163" t="s">
         <v>805</v>
       </c>
-      <c r="H17" s="148"/>
-      <c r="I17" s="149"/>
+      <c r="H17" s="161"/>
+      <c r="I17" s="162"/>
     </row>
     <row r="18" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A18" s="96">
@@ -16631,15 +16633,15 @@
       <c r="D18" s="91" t="s">
         <v>799</v>
       </c>
-      <c r="E18" s="152" t="s">
+      <c r="E18" s="163" t="s">
         <v>804</v>
       </c>
-      <c r="F18" s="145"/>
-      <c r="G18" s="152" t="s">
+      <c r="F18" s="160"/>
+      <c r="G18" s="163" t="s">
         <v>807</v>
       </c>
-      <c r="H18" s="148"/>
-      <c r="I18" s="149"/>
+      <c r="H18" s="161"/>
+      <c r="I18" s="162"/>
     </row>
     <row r="19" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A19" s="96">
@@ -16654,15 +16656,15 @@
       <c r="D19" s="91" t="s">
         <v>809</v>
       </c>
-      <c r="E19" s="152" t="s">
+      <c r="E19" s="163" t="s">
         <v>810</v>
       </c>
-      <c r="F19" s="145"/>
-      <c r="G19" s="152" t="s">
+      <c r="F19" s="160"/>
+      <c r="G19" s="163" t="s">
         <v>811</v>
       </c>
-      <c r="H19" s="148"/>
-      <c r="I19" s="149"/>
+      <c r="H19" s="161"/>
+      <c r="I19" s="162"/>
       <c r="K19" s="81" t="s">
         <v>812</v>
       </c>
@@ -16674,11 +16676,11 @@
       <c r="B20" s="97"/>
       <c r="C20" s="97"/>
       <c r="D20" s="97"/>
-      <c r="E20" s="144"/>
-      <c r="F20" s="145"/>
-      <c r="G20" s="144"/>
-      <c r="H20" s="148"/>
-      <c r="I20" s="149"/>
+      <c r="E20" s="164"/>
+      <c r="F20" s="160"/>
+      <c r="G20" s="164"/>
+      <c r="H20" s="161"/>
+      <c r="I20" s="162"/>
     </row>
     <row r="21" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A21" s="96">
@@ -16687,11 +16689,11 @@
       <c r="B21" s="97"/>
       <c r="C21" s="97"/>
       <c r="D21" s="97"/>
-      <c r="E21" s="144"/>
-      <c r="F21" s="145"/>
-      <c r="G21" s="144"/>
-      <c r="H21" s="148"/>
-      <c r="I21" s="149"/>
+      <c r="E21" s="164"/>
+      <c r="F21" s="160"/>
+      <c r="G21" s="164"/>
+      <c r="H21" s="161"/>
+      <c r="I21" s="162"/>
       <c r="K21" s="81" t="s">
         <v>813</v>
       </c>
@@ -16703,11 +16705,11 @@
       <c r="B22" s="97"/>
       <c r="C22" s="97"/>
       <c r="D22" s="97"/>
-      <c r="E22" s="144"/>
-      <c r="F22" s="145"/>
-      <c r="G22" s="144"/>
-      <c r="H22" s="148"/>
-      <c r="I22" s="149"/>
+      <c r="E22" s="164"/>
+      <c r="F22" s="160"/>
+      <c r="G22" s="164"/>
+      <c r="H22" s="161"/>
+      <c r="I22" s="162"/>
     </row>
     <row r="23" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A23" s="96">
@@ -16716,11 +16718,11 @@
       <c r="B23" s="97"/>
       <c r="C23" s="97"/>
       <c r="D23" s="97"/>
-      <c r="E23" s="144"/>
-      <c r="F23" s="145"/>
-      <c r="G23" s="144"/>
-      <c r="H23" s="148"/>
-      <c r="I23" s="149"/>
+      <c r="E23" s="164"/>
+      <c r="F23" s="160"/>
+      <c r="G23" s="164"/>
+      <c r="H23" s="161"/>
+      <c r="I23" s="162"/>
     </row>
     <row r="24" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A24" s="96">
@@ -16729,11 +16731,11 @@
       <c r="B24" s="97"/>
       <c r="C24" s="97"/>
       <c r="D24" s="97"/>
-      <c r="E24" s="144"/>
-      <c r="F24" s="145"/>
-      <c r="G24" s="144"/>
-      <c r="H24" s="148"/>
-      <c r="I24" s="149"/>
+      <c r="E24" s="164"/>
+      <c r="F24" s="160"/>
+      <c r="G24" s="164"/>
+      <c r="H24" s="161"/>
+      <c r="I24" s="162"/>
     </row>
     <row r="25" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A25" s="96">
@@ -16742,11 +16744,11 @@
       <c r="B25" s="97"/>
       <c r="C25" s="97"/>
       <c r="D25" s="97"/>
-      <c r="E25" s="144"/>
-      <c r="F25" s="145"/>
-      <c r="G25" s="144"/>
-      <c r="H25" s="148"/>
-      <c r="I25" s="149"/>
+      <c r="E25" s="164"/>
+      <c r="F25" s="160"/>
+      <c r="G25" s="164"/>
+      <c r="H25" s="161"/>
+      <c r="I25" s="162"/>
     </row>
     <row r="26" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="98">
@@ -16755,11 +16757,11 @@
       <c r="B26" s="94"/>
       <c r="C26" s="94"/>
       <c r="D26" s="94"/>
-      <c r="E26" s="146"/>
-      <c r="F26" s="147"/>
-      <c r="G26" s="146"/>
+      <c r="E26" s="165"/>
+      <c r="F26" s="148"/>
+      <c r="G26" s="165"/>
       <c r="H26" s="150"/>
-      <c r="I26" s="151"/>
+      <c r="I26" s="152"/>
     </row>
     <row r="27" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="28" spans="1:11" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -17737,16 +17739,14 @@
     <row r="1000" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   </sheetData>
   <mergeCells count="30">
-    <mergeCell ref="A1:I1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="D2:G2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="A4:I4"/>
-    <mergeCell ref="K6:Q6"/>
-    <mergeCell ref="K7:Q7"/>
-    <mergeCell ref="A15:I15"/>
-    <mergeCell ref="E16:F16"/>
-    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="E23:F23"/>
+    <mergeCell ref="E24:F24"/>
+    <mergeCell ref="E25:F25"/>
+    <mergeCell ref="E26:F26"/>
+    <mergeCell ref="G23:I23"/>
+    <mergeCell ref="G24:I24"/>
+    <mergeCell ref="G25:I25"/>
+    <mergeCell ref="G26:I26"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="G17:I17"/>
     <mergeCell ref="E18:F18"/>
@@ -17759,14 +17759,16 @@
     <mergeCell ref="E21:F21"/>
     <mergeCell ref="G21:I21"/>
     <mergeCell ref="G22:I22"/>
-    <mergeCell ref="E23:F23"/>
-    <mergeCell ref="E24:F24"/>
-    <mergeCell ref="E25:F25"/>
-    <mergeCell ref="E26:F26"/>
-    <mergeCell ref="G23:I23"/>
-    <mergeCell ref="G24:I24"/>
-    <mergeCell ref="G25:I25"/>
-    <mergeCell ref="G26:I26"/>
+    <mergeCell ref="K6:Q6"/>
+    <mergeCell ref="K7:Q7"/>
+    <mergeCell ref="A15:I15"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="G16:I16"/>
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:B2"/>
+    <mergeCell ref="D2:G2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="A4:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0" footer="0"/>
   <pageSetup orientation="landscape"/>
@@ -19347,7 +19349,7 @@
       <c r="B2" s="168" t="s">
         <v>824</v>
       </c>
-      <c r="C2" s="145"/>
+      <c r="C2" s="160"/>
       <c r="O2" s="81" t="s">
         <v>825</v>
       </c>
@@ -20561,8 +20563,8 @@
       <c r="A3" s="168" t="s">
         <v>857</v>
       </c>
-      <c r="B3" s="148"/>
-      <c r="C3" s="145"/>
+      <c r="B3" s="161"/>
+      <c r="C3" s="160"/>
     </row>
     <row r="4" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="120" t="s">
@@ -20571,7 +20573,7 @@
       <c r="B4" s="170" t="s">
         <v>858</v>
       </c>
-      <c r="C4" s="145"/>
+      <c r="C4" s="160"/>
     </row>
     <row r="5" spans="1:10" ht="96" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="121" t="s">
@@ -20580,7 +20582,7 @@
       <c r="B5" s="169" t="s">
         <v>860</v>
       </c>
-      <c r="C5" s="145"/>
+      <c r="C5" s="160"/>
     </row>
     <row r="6" spans="1:10" ht="64.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A6" s="121" t="s">
@@ -20589,7 +20591,7 @@
       <c r="B6" s="169" t="s">
         <v>862</v>
       </c>
-      <c r="C6" s="145"/>
+      <c r="C6" s="160"/>
     </row>
     <row r="7" spans="1:10" ht="67.5" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A7" s="121" t="s">
@@ -20598,7 +20600,7 @@
       <c r="B7" s="169" t="s">
         <v>864</v>
       </c>
-      <c r="C7" s="145"/>
+      <c r="C7" s="160"/>
     </row>
     <row r="8" spans="1:10" ht="72.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A8" s="121" t="s">
@@ -20607,7 +20609,7 @@
       <c r="B8" s="169" t="s">
         <v>866</v>
       </c>
-      <c r="C8" s="145"/>
+      <c r="C8" s="160"/>
     </row>
     <row r="9" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="10" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.2"/>
@@ -21635,8 +21637,8 @@
       <c r="B2" s="171" t="s">
         <v>867</v>
       </c>
-      <c r="C2" s="160"/>
-      <c r="D2" s="161"/>
+      <c r="C2" s="145"/>
+      <c r="D2" s="146"/>
       <c r="J2" s="81" t="s">
         <v>825</v>
       </c>
@@ -24220,8 +24222,8 @@
       <c r="A5" s="170" t="s">
         <v>900</v>
       </c>
-      <c r="B5" s="148"/>
-      <c r="C5" s="145"/>
+      <c r="B5" s="161"/>
+      <c r="C5" s="160"/>
     </row>
     <row r="6" spans="1:10" ht="14.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="120" t="s">

</xml_diff>